<commit_message>
gen pakeitimai, saraso korekcijos
</commit_message>
<xml_diff>
--- a/Apdailos kodo gen exceliai/Apdailos kodo generacija - Test versija3.xlsx
+++ b/Apdailos kodo gen exceliai/Apdailos kodo generacija - Test versija3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://svenheimuab-my.sharepoint.com/personal/ignven_svenheim_lt/Documents/Desktop/Apdailos kodo gen/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://svenheimuab-my.sharepoint.com/personal/ignven_svenheim_lt/Documents/Desktop/CODE/apdailos-kodo-generatorius/Apdailos kodo gen exceliai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="8_{6EEF2F4A-8834-4DAF-B727-7DA66127EA47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87A603CE-2081-42FB-897E-C552FECF4E5C}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="8_{6EEF2F4A-8834-4DAF-B727-7DA66127EA47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6754F58C-74BA-4594-B6F2-52D4565802BA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Generatorius" sheetId="1" r:id="rId1"/>
@@ -1982,6 +1982,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1991,6 +1997,78 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2029,84 +2107,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2123,10 +2123,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2580,11 +2576,11 @@
         <v>=</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>207</v>
+        <v>120</v>
       </c>
       <c r="D13" s="82" t="str">
         <f>IF(C13="",CONCATENATE(A13, B13,  C13, "",),CONCATENATE(A13, B13,  C13, " ",))</f>
-        <v xml:space="preserve">E=S2005-G70Y </v>
+        <v xml:space="preserve">E=S0500-N </v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -3394,11 +3390,11 @@
   <sheetData>
     <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="95" t="s">
+      <c r="B2" s="121" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="96"/>
-      <c r="D2" s="97"/>
+      <c r="C2" s="122"/>
+      <c r="D2" s="123"/>
       <c r="I2" s="31" t="s">
         <v>126</v>
       </c>
@@ -3556,14 +3552,14 @@
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="98" t="s">
+      <c r="B12" s="124" t="s">
         <v>148</v>
       </c>
-      <c r="C12" s="98"/>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98"/>
-      <c r="G12" s="98"/>
+      <c r="C12" s="124"/>
+      <c r="D12" s="124"/>
+      <c r="E12" s="124"/>
+      <c r="F12" s="124"/>
+      <c r="G12" s="124"/>
       <c r="I12" s="47"/>
       <c r="J12" s="48"/>
     </row>
@@ -3584,15 +3580,15 @@
       <c r="B15" s="50" t="s">
         <v>150</v>
       </c>
-      <c r="C15" s="99" t="s">
+      <c r="C15" s="125" t="s">
         <v>151</v>
       </c>
-      <c r="D15" s="100"/>
-      <c r="E15" s="100"/>
-      <c r="F15" s="100"/>
-      <c r="G15" s="100"/>
-      <c r="H15" s="100"/>
-      <c r="I15" s="101"/>
+      <c r="D15" s="126"/>
+      <c r="E15" s="126"/>
+      <c r="F15" s="126"/>
+      <c r="G15" s="126"/>
+      <c r="H15" s="126"/>
+      <c r="I15" s="127"/>
       <c r="J15" s="51" t="s">
         <v>152</v>
       </c>
@@ -3601,15 +3597,15 @@
       <c r="B16" s="52">
         <v>1</v>
       </c>
-      <c r="C16" s="110" t="s">
+      <c r="C16" s="97" t="s">
         <v>153</v>
       </c>
-      <c r="D16" s="111"/>
-      <c r="E16" s="111"/>
-      <c r="F16" s="111"/>
-      <c r="G16" s="111"/>
-      <c r="H16" s="111"/>
-      <c r="I16" s="112"/>
+      <c r="D16" s="98"/>
+      <c r="E16" s="98"/>
+      <c r="F16" s="98"/>
+      <c r="G16" s="98"/>
+      <c r="H16" s="98"/>
+      <c r="I16" s="99"/>
       <c r="J16" s="53" t="s">
         <v>137</v>
       </c>
@@ -3618,15 +3614,15 @@
       <c r="B17" s="54">
         <v>2</v>
       </c>
-      <c r="C17" s="92" t="s">
+      <c r="C17" s="94" t="s">
         <v>193</v>
       </c>
-      <c r="D17" s="93"/>
-      <c r="E17" s="93"/>
-      <c r="F17" s="93"/>
-      <c r="G17" s="93"/>
-      <c r="H17" s="93"/>
-      <c r="I17" s="94"/>
+      <c r="D17" s="95"/>
+      <c r="E17" s="95"/>
+      <c r="F17" s="95"/>
+      <c r="G17" s="95"/>
+      <c r="H17" s="95"/>
+      <c r="I17" s="96"/>
       <c r="J17" s="55" t="s">
         <v>154</v>
       </c>
@@ -3635,15 +3631,15 @@
       <c r="B18" s="56">
         <v>3</v>
       </c>
-      <c r="C18" s="92" t="s">
+      <c r="C18" s="94" t="s">
         <v>155</v>
       </c>
-      <c r="D18" s="93"/>
-      <c r="E18" s="93"/>
-      <c r="F18" s="93"/>
-      <c r="G18" s="93"/>
-      <c r="H18" s="93"/>
-      <c r="I18" s="94"/>
+      <c r="D18" s="95"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="95"/>
+      <c r="G18" s="95"/>
+      <c r="H18" s="95"/>
+      <c r="I18" s="96"/>
       <c r="J18" s="55" t="s">
         <v>156</v>
       </c>
@@ -3652,15 +3648,15 @@
       <c r="B19" s="54">
         <v>4</v>
       </c>
-      <c r="C19" s="102" t="s">
+      <c r="C19" s="128" t="s">
         <v>157</v>
       </c>
-      <c r="D19" s="103"/>
-      <c r="E19" s="103"/>
-      <c r="F19" s="103"/>
-      <c r="G19" s="103"/>
-      <c r="H19" s="103"/>
-      <c r="I19" s="104"/>
+      <c r="D19" s="129"/>
+      <c r="E19" s="129"/>
+      <c r="F19" s="129"/>
+      <c r="G19" s="129"/>
+      <c r="H19" s="129"/>
+      <c r="I19" s="130"/>
       <c r="J19" s="37" t="s">
         <v>158</v>
       </c>
@@ -3669,15 +3665,15 @@
       <c r="B20" s="54">
         <v>5</v>
       </c>
-      <c r="C20" s="102" t="s">
+      <c r="C20" s="128" t="s">
         <v>159</v>
       </c>
-      <c r="D20" s="103"/>
-      <c r="E20" s="103"/>
-      <c r="F20" s="103"/>
-      <c r="G20" s="103"/>
-      <c r="H20" s="103"/>
-      <c r="I20" s="104"/>
+      <c r="D20" s="129"/>
+      <c r="E20" s="129"/>
+      <c r="F20" s="129"/>
+      <c r="G20" s="129"/>
+      <c r="H20" s="129"/>
+      <c r="I20" s="130"/>
       <c r="J20" s="37" t="s">
         <v>160</v>
       </c>
@@ -3686,15 +3682,15 @@
       <c r="B21" s="54">
         <v>6</v>
       </c>
-      <c r="C21" s="105" t="s">
+      <c r="C21" s="131" t="s">
         <v>161</v>
       </c>
-      <c r="D21" s="106"/>
-      <c r="E21" s="106"/>
-      <c r="F21" s="106"/>
-      <c r="G21" s="106"/>
-      <c r="H21" s="106"/>
-      <c r="I21" s="107"/>
+      <c r="D21" s="132"/>
+      <c r="E21" s="132"/>
+      <c r="F21" s="132"/>
+      <c r="G21" s="132"/>
+      <c r="H21" s="132"/>
+      <c r="I21" s="133"/>
       <c r="J21" s="57" t="s">
         <v>162</v>
       </c>
@@ -3703,15 +3699,15 @@
       <c r="B22" s="54">
         <v>7</v>
       </c>
-      <c r="C22" s="105" t="s">
+      <c r="C22" s="131" t="s">
         <v>163</v>
       </c>
-      <c r="D22" s="106"/>
-      <c r="E22" s="106"/>
-      <c r="F22" s="106"/>
-      <c r="G22" s="106"/>
-      <c r="H22" s="106"/>
-      <c r="I22" s="107"/>
+      <c r="D22" s="132"/>
+      <c r="E22" s="132"/>
+      <c r="F22" s="132"/>
+      <c r="G22" s="132"/>
+      <c r="H22" s="132"/>
+      <c r="I22" s="133"/>
       <c r="J22" s="37" t="s">
         <v>164</v>
       </c>
@@ -3720,15 +3716,15 @@
       <c r="B23" s="54">
         <v>8</v>
       </c>
-      <c r="C23" s="102" t="s">
+      <c r="C23" s="128" t="s">
         <v>165</v>
       </c>
-      <c r="D23" s="103"/>
-      <c r="E23" s="103"/>
-      <c r="F23" s="103"/>
-      <c r="G23" s="103"/>
-      <c r="H23" s="103"/>
-      <c r="I23" s="104"/>
+      <c r="D23" s="129"/>
+      <c r="E23" s="129"/>
+      <c r="F23" s="129"/>
+      <c r="G23" s="129"/>
+      <c r="H23" s="129"/>
+      <c r="I23" s="130"/>
       <c r="J23" s="37" t="s">
         <v>7</v>
       </c>
@@ -3737,15 +3733,15 @@
       <c r="B24" s="54">
         <v>9</v>
       </c>
-      <c r="C24" s="92" t="s">
+      <c r="C24" s="94" t="s">
         <v>166</v>
       </c>
-      <c r="D24" s="93"/>
-      <c r="E24" s="93"/>
-      <c r="F24" s="93"/>
-      <c r="G24" s="93"/>
-      <c r="H24" s="93"/>
-      <c r="I24" s="94"/>
+      <c r="D24" s="95"/>
+      <c r="E24" s="95"/>
+      <c r="F24" s="95"/>
+      <c r="G24" s="95"/>
+      <c r="H24" s="95"/>
+      <c r="I24" s="96"/>
       <c r="J24" s="55" t="s">
         <v>167</v>
       </c>
@@ -3754,15 +3750,15 @@
       <c r="B25" s="54">
         <v>10</v>
       </c>
-      <c r="C25" s="92" t="s">
+      <c r="C25" s="94" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="93"/>
-      <c r="E25" s="93"/>
-      <c r="F25" s="93"/>
-      <c r="G25" s="93"/>
-      <c r="H25" s="93"/>
-      <c r="I25" s="94"/>
+      <c r="D25" s="95"/>
+      <c r="E25" s="95"/>
+      <c r="F25" s="95"/>
+      <c r="G25" s="95"/>
+      <c r="H25" s="95"/>
+      <c r="I25" s="96"/>
       <c r="J25" s="55" t="s">
         <v>167</v>
       </c>
@@ -3771,15 +3767,15 @@
       <c r="B26" s="54">
         <v>11</v>
       </c>
-      <c r="C26" s="92" t="s">
+      <c r="C26" s="94" t="s">
         <v>192</v>
       </c>
-      <c r="D26" s="93"/>
-      <c r="E26" s="93"/>
-      <c r="F26" s="93"/>
-      <c r="G26" s="93"/>
-      <c r="H26" s="93"/>
-      <c r="I26" s="94"/>
+      <c r="D26" s="95"/>
+      <c r="E26" s="95"/>
+      <c r="F26" s="95"/>
+      <c r="G26" s="95"/>
+      <c r="H26" s="95"/>
+      <c r="I26" s="96"/>
       <c r="J26" s="55" t="s">
         <v>191</v>
       </c>
@@ -3788,15 +3784,15 @@
       <c r="B27" s="54">
         <v>12</v>
       </c>
-      <c r="C27" s="92" t="s">
+      <c r="C27" s="94" t="s">
         <v>169</v>
       </c>
-      <c r="D27" s="93"/>
-      <c r="E27" s="93"/>
-      <c r="F27" s="93"/>
-      <c r="G27" s="93"/>
-      <c r="H27" s="93"/>
-      <c r="I27" s="94"/>
+      <c r="D27" s="95"/>
+      <c r="E27" s="95"/>
+      <c r="F27" s="95"/>
+      <c r="G27" s="95"/>
+      <c r="H27" s="95"/>
+      <c r="I27" s="96"/>
       <c r="J27" s="55" t="s">
         <v>170</v>
       </c>
@@ -3805,15 +3801,15 @@
       <c r="B28" s="58">
         <v>13</v>
       </c>
-      <c r="C28" s="121" t="s">
+      <c r="C28" s="108" t="s">
         <v>171</v>
       </c>
-      <c r="D28" s="122"/>
-      <c r="E28" s="122"/>
-      <c r="F28" s="122"/>
-      <c r="G28" s="122"/>
-      <c r="H28" s="122"/>
-      <c r="I28" s="123"/>
+      <c r="D28" s="109"/>
+      <c r="E28" s="109"/>
+      <c r="F28" s="109"/>
+      <c r="G28" s="109"/>
+      <c r="H28" s="109"/>
+      <c r="I28" s="110"/>
       <c r="J28" s="59" t="s">
         <v>7</v>
       </c>
@@ -3821,12 +3817,12 @@
     <row r="29" spans="2:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="2:10" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="31" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="124" t="s">
+      <c r="B31" s="111" t="s">
         <v>172</v>
       </c>
-      <c r="C31" s="125"/>
-      <c r="D31" s="126"/>
-      <c r="E31" s="127"/>
+      <c r="C31" s="112"/>
+      <c r="D31" s="113"/>
+      <c r="E31" s="114"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B32" s="57">
@@ -3835,10 +3831,10 @@
       <c r="C32" s="60" t="s">
         <v>173</v>
       </c>
-      <c r="D32" s="128" t="s">
+      <c r="D32" s="115" t="s">
         <v>174</v>
       </c>
-      <c r="E32" s="129"/>
+      <c r="E32" s="116"/>
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B33" s="37">
@@ -3847,10 +3843,10 @@
       <c r="C33" s="61" t="s">
         <v>175</v>
       </c>
-      <c r="D33" s="130" t="s">
+      <c r="D33" s="117" t="s">
         <v>176</v>
       </c>
-      <c r="E33" s="131"/>
+      <c r="E33" s="118"/>
       <c r="T33" s="62"/>
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.25">
@@ -3860,10 +3856,10 @@
       <c r="C34" s="61" t="s">
         <v>177</v>
       </c>
-      <c r="D34" s="130" t="s">
+      <c r="D34" s="117" t="s">
         <v>178</v>
       </c>
-      <c r="E34" s="131"/>
+      <c r="E34" s="118"/>
       <c r="H34" s="62"/>
     </row>
     <row r="35" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3873,73 +3869,85 @@
       <c r="C35" s="63" t="s">
         <v>179</v>
       </c>
-      <c r="D35" s="132" t="s">
+      <c r="D35" s="119" t="s">
         <v>180</v>
       </c>
-      <c r="E35" s="133"/>
+      <c r="E35" s="120"/>
     </row>
     <row r="36" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="37" spans="2:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C37" s="113" t="s">
+      <c r="C37" s="100" t="s">
         <v>181</v>
       </c>
-      <c r="D37" s="114"/>
-      <c r="E37" s="115"/>
+      <c r="D37" s="101"/>
+      <c r="E37" s="102"/>
     </row>
     <row r="38" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C38" s="116" t="s">
+      <c r="C38" s="103" t="s">
         <v>182</v>
       </c>
-      <c r="D38" s="117"/>
-      <c r="E38" s="118"/>
+      <c r="D38" s="104"/>
+      <c r="E38" s="105"/>
     </row>
     <row r="39" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C39" s="64" t="s">
         <v>183</v>
       </c>
-      <c r="D39" s="119" t="s">
+      <c r="D39" s="106" t="s">
         <v>184</v>
       </c>
-      <c r="E39" s="120"/>
+      <c r="E39" s="107"/>
     </row>
     <row r="40" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C40" s="65" t="s">
         <v>185</v>
       </c>
-      <c r="D40" s="119" t="s">
+      <c r="D40" s="106" t="s">
         <v>186</v>
       </c>
-      <c r="E40" s="120"/>
+      <c r="E40" s="107"/>
     </row>
     <row r="41" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C41" s="65" t="s">
         <v>187</v>
       </c>
-      <c r="D41" s="119" t="s">
+      <c r="D41" s="106" t="s">
         <v>188</v>
       </c>
-      <c r="E41" s="120"/>
+      <c r="E41" s="107"/>
     </row>
     <row r="42" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C42" s="65" t="s">
         <v>179</v>
       </c>
-      <c r="D42" s="119" t="s">
+      <c r="D42" s="106" t="s">
         <v>189</v>
       </c>
-      <c r="E42" s="120"/>
+      <c r="E42" s="107"/>
     </row>
     <row r="43" spans="2:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C43" s="66" t="s">
         <v>173</v>
       </c>
-      <c r="D43" s="108" t="s">
+      <c r="D43" s="92" t="s">
         <v>190</v>
       </c>
-      <c r="E43" s="109"/>
+      <c r="E43" s="93"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C19:I19"/>
+    <mergeCell ref="C20:I20"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C23:I23"/>
+    <mergeCell ref="C24:I24"/>
+    <mergeCell ref="C25:I25"/>
+    <mergeCell ref="C26:I26"/>
     <mergeCell ref="D43:E43"/>
     <mergeCell ref="C17:I17"/>
     <mergeCell ref="C16:I16"/>
@@ -3956,18 +3964,6 @@
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="D35:E35"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="C19:I19"/>
-    <mergeCell ref="C20:I20"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="C22:I22"/>
-    <mergeCell ref="C23:I23"/>
-    <mergeCell ref="C24:I24"/>
-    <mergeCell ref="C25:I25"/>
-    <mergeCell ref="C26:I26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>